<commit_message>
Add contacts index to app routing and update file sharing template
- Added 'contacts' index to the application routing for improved navigation.
- Removed access logs display from the file sharing settings template to streamline the user interface.
- Updated the binary file 'beispiel_staende.xlsx' in the assessment static files.
</commit_message>
<xml_diff>
--- a/app/static/assessment/beispiel_staende.xlsx
+++ b/app/static/assessment/beispiel_staende.xlsx
@@ -1,26 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ermat\Documents\Sommerfest\V_1_0_4 - beta\static\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ermat\Documents\GitHub\Prismateams_web\app\static\assessment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88264A4A-BED4-4121-8AA8-A39A2F75D927}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F414824-7C9A-442B-A784-77FFD3C36BF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2685" yWindow="2685" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Stand Anlegung" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>Standname</t>
   </si>
@@ -56,6 +61,18 @@
   </si>
   <si>
     <t>Foyer</t>
+  </si>
+  <si>
+    <t>Standtyp</t>
+  </si>
+  <si>
+    <t>Essen</t>
+  </si>
+  <si>
+    <t>Aktivität</t>
+  </si>
+  <si>
+    <t>Kombi</t>
   </si>
 </sst>
 </file>
@@ -317,10 +334,10 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -330,8 +347,11 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="D1" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -341,8 +361,11 @@
       <c r="C2" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="D2" s="1" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -352,8 +375,11 @@
       <c r="C3" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="D3" s="1" t="s">
+        <v>14</v>
+      </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>9</v>
       </c>
@@ -362,6 +388,9 @@
       </c>
       <c r="C4" s="1" t="s">
         <v>11</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>